<commit_message>
update design changes 5
</commit_message>
<xml_diff>
--- a/src/main/resources/static/xl-folder/Liabilities_Summary.xlsx
+++ b/src/main/resources/static/xl-folder/Liabilities_Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A78A510-5778-41EE-808B-B41F7D013BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2699FD4A-A47D-4448-85EF-92E92C452F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
-  <si>
-    <t>Date</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
   <si>
     <t>Liabilities summary</t>
   </si>
@@ -171,25 +168,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
+  <numFmts count="3">
     <numFmt numFmtId="165" formatCode="\₹#,##0;&quot;(₹&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.00%;\-0.00%;;@"/>
     <numFmt numFmtId="167" formatCode="0.00;\-0.00;\-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <charset val="1"/>
     </font>
     <font>
@@ -311,55 +300,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -624,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -635,454 +619,437 @@
     <col min="7" max="7" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="e">
-        <f>"Liabilities summary for "&amp;#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="7"/>
-    </row>
-    <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="1" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="8" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D13" si="0">ROUND(B3*C3/12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
+        <f t="shared" ref="E3:E13" si="1">ROUND(B3*C3,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="10">
-        <v>0</v>
-      </c>
-      <c r="C6" s="11">
-        <v>0</v>
-      </c>
-      <c r="D6" s="12">
-        <f t="shared" ref="D6:D16" si="0">ROUND(B6*C6/12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="12">
-        <f t="shared" ref="E6:E16" si="1">ROUND(B6*C6,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="10">
+      <c r="B4" s="3">
         <v>543255</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C4" s="4">
         <v>0.12</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D4" s="5">
         <f t="shared" si="0"/>
         <v>5433</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E4" s="5">
         <f t="shared" si="1"/>
         <v>65191</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="10">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3">
         <v>1952355</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C5" s="4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D5" s="5">
         <f t="shared" si="0"/>
         <v>22777</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E5" s="5">
         <f t="shared" si="1"/>
         <v>273330</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="10">
-        <v>0</v>
-      </c>
-      <c r="C9" s="11">
-        <v>0</v>
-      </c>
-      <c r="D9" s="12">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>0</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="5">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="10">
-        <v>0</v>
-      </c>
-      <c r="C10" s="11">
-        <v>0</v>
-      </c>
-      <c r="D10" s="12">
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="5">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="10">
-        <v>0</v>
-      </c>
-      <c r="C11" s="11">
-        <v>0</v>
-      </c>
-      <c r="D11" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E11" s="12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="10">
-        <v>0</v>
-      </c>
-      <c r="C12" s="11">
-        <v>0</v>
-      </c>
-      <c r="D12" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E12" s="12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+      <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="10">
-        <v>0</v>
-      </c>
-      <c r="C13" s="11">
-        <v>0</v>
-      </c>
-      <c r="D13" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E13" s="12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="10">
+      <c r="B11" s="3">
         <v>380000</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C11" s="4">
         <v>9.7500000000000003E-2</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D11" s="5">
         <f t="shared" si="0"/>
         <v>3088</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E11" s="5">
         <f t="shared" si="1"/>
         <v>37050</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="10">
-        <v>0</v>
-      </c>
-      <c r="C15" s="11">
-        <v>0</v>
-      </c>
-      <c r="D15" s="12">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E12" s="5">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="10">
-        <v>0</v>
-      </c>
-      <c r="C16" s="11">
-        <v>0</v>
-      </c>
-      <c r="D16" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E16" s="12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B14" s="7">
+        <f>SUM(B3:B13)</f>
+        <v>2875610</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D3:D13)</f>
+        <v>31298</v>
+      </c>
+      <c r="E14" s="7">
+        <f>ROUND(SUMPRODUCT(B3:B13,C3:C13),0)</f>
+        <v>375570</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="14">
-        <f>SUM(B6:B16)</f>
-        <v>2875610</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="14">
-        <f>SUM(D6:D16)</f>
-        <v>31298</v>
-      </c>
-      <c r="E17" s="14">
-        <f>ROUND(SUMPRODUCT(B6:B16,C6:C16),0)</f>
-        <v>375570</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="s">
+      <c r="B17" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="C17" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+    </row>
+    <row r="18" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+      <c r="B18" s="12">
+        <f>ROUND(E14/B14*100,2)</f>
+        <v>13.06</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+    </row>
+    <row r="19" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="12">
+        <f>IF(B25=0,"",ROUND(E14/B25*100,2))</f>
+        <v>31.3</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+    </row>
+    <row r="20" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="12">
+        <f>IF(B27=0,"",ROUND(B14/B27*100,2))</f>
+        <v>31.95</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
     </row>
     <row r="21" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="19">
-        <f>ROUND(E17/B17*100,2)</f>
-        <v>13.06</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="12">
+        <f>IF(B28=0,"",ROUND(E14/B28*100,2))</f>
+        <v>150.22999999999999</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
     </row>
     <row r="22" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="12">
+        <f>IF(B25=0,"",ROUND(B26/B25*100,2))</f>
         <v>25</v>
       </c>
-      <c r="B22" s="19">
-        <f>IF(B28=0,"",ROUND(E17/B28*100,2))</f>
-        <v>31.3</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="19">
-        <f>IF(B30=0,"",ROUND(B17/B30*100,2))</f>
-        <v>31.95</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="19">
-        <f>IF(B31=0,"",ROUND(E17/B31*100,2))</f>
-        <v>150.22999999999999</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="18" t="s">
+      <c r="C22" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="19">
-        <f>IF(B28=0,"",ROUND(B29/B28*100,2))</f>
-        <v>25</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+    </row>
+    <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="27" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="B25" s="3">
+        <v>1200000</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+    </row>
+    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="3">
+        <v>300000</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+    </row>
+    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="3">
+        <v>9000000</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
     </row>
     <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="10">
-        <v>1200000</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" s="10">
-        <v>300000</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="10">
-        <v>9000000</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="A28" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
+      <c r="B28" s="3">
+        <v>250000</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="10">
-        <v>250000</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+    </row>
+    <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-    </row>
-    <row r="34" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="A27:E27"/>
+  <mergeCells count="14">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="A31:E31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>